<commit_message>
pilot-108: поиск+суждения 2026-08-27 (run 33049218185)
</commit_message>
<xml_diff>
--- a/output/Пилот108_2026-08-27.xlsx
+++ b/output/Пилот108_2026-08-27.xlsx
@@ -647,7 +647,9 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="inlineStr"/>
-      <c r="W2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -888,7 +890,9 @@
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="2" t="inlineStr"/>
+      <c r="W5" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1014,27 +1018,57 @@
           <t>Казань</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>karsar.ru</t>
+        </is>
+      </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Казань (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr"/>
-      <c r="U7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1283,7 +1317,9 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="inlineStr"/>
-      <c r="W10" s="2" t="inlineStr"/>
+      <c r="W10" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1350,7 +1386,9 @@
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="inlineStr"/>
-      <c r="W11" s="2" t="inlineStr"/>
+      <c r="W11" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1417,7 +1455,9 @@
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="inlineStr"/>
-      <c r="W12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1579,7 +1619,9 @@
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="inlineStr"/>
-      <c r="W14" s="2" t="inlineStr"/>
+      <c r="W14" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1820,7 +1862,9 @@
       <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="inlineStr"/>
-      <c r="W17" s="2" t="inlineStr"/>
+      <c r="W17" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1867,27 +1911,57 @@
           <t>Краснодар</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>compressor-borec.ru</t>
+        </is>
+      </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Краснодар (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="inlineStr"/>
-      <c r="T18" s="2" t="inlineStr"/>
-      <c r="U18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V18" s="2" t="inlineStr"/>
-      <c r="W18" s="2" t="inlineStr"/>
+      <c r="W18" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1954,7 +2028,9 @@
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="inlineStr"/>
-      <c r="W19" s="2" t="inlineStr"/>
+      <c r="W19" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2306,7 +2382,9 @@
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="inlineStr"/>
-      <c r="W23" s="2" t="inlineStr"/>
+      <c r="W23" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2373,7 +2451,9 @@
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="inlineStr"/>
-      <c r="W24" s="2" t="inlineStr"/>
+      <c r="W24" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2527,7 +2607,9 @@
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="inlineStr"/>
-      <c r="W26" s="2" t="inlineStr"/>
+      <c r="W26" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2594,7 +2676,9 @@
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="inlineStr"/>
-      <c r="W27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2661,7 +2745,9 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="inlineStr"/>
-      <c r="W28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2728,7 +2814,9 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="inlineStr"/>
-      <c r="W29" s="2" t="inlineStr"/>
+      <c r="W29" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2787,7 +2875,9 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="inlineStr"/>
-      <c r="W30" s="2" t="inlineStr"/>
+      <c r="W30" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2830,23 +2920,57 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>cnmt.ru</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 5408307710 найден на сайте</t>
+        </is>
+      </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr"/>
-      <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Консультация флеболога и УЗИ вен за»</t>
+        </is>
+      </c>
       <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="inlineStr"/>
-      <c r="U31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V31" s="2" t="inlineStr"/>
-      <c r="W31" s="2" t="inlineStr"/>
+      <c r="W31" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2905,7 +3029,9 @@
       <c r="T32" s="2" t="inlineStr"/>
       <c r="U32" s="2" t="inlineStr"/>
       <c r="V32" s="2" t="inlineStr"/>
-      <c r="W32" s="2" t="inlineStr"/>
+      <c r="W32" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2948,23 +3074,57 @@
           <t>Краснодар</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>samson23.ru</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Краснодар (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S33" s="2" t="inlineStr"/>
-      <c r="T33" s="2" t="inlineStr"/>
-      <c r="U33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V33" s="2" t="inlineStr"/>
-      <c r="W33" s="2" t="inlineStr"/>
+      <c r="W33" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3023,7 +3183,9 @@
       <c r="T34" s="2" t="inlineStr"/>
       <c r="U34" s="2" t="inlineStr"/>
       <c r="V34" s="2" t="inlineStr"/>
-      <c r="W34" s="2" t="inlineStr"/>
+      <c r="W34" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3082,7 +3244,9 @@
       <c r="T35" s="2" t="inlineStr"/>
       <c r="U35" s="2" t="inlineStr"/>
       <c r="V35" s="2" t="inlineStr"/>
-      <c r="W35" s="2" t="inlineStr"/>
+      <c r="W35" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3315,7 +3479,9 @@
       <c r="T38" s="2" t="inlineStr"/>
       <c r="U38" s="2" t="inlineStr"/>
       <c r="V38" s="2" t="inlineStr"/>
-      <c r="W38" s="2" t="inlineStr"/>
+      <c r="W38" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3374,7 +3540,9 @@
       <c r="T39" s="2" t="inlineStr"/>
       <c r="U39" s="2" t="inlineStr"/>
       <c r="V39" s="2" t="inlineStr"/>
-      <c r="W39" s="2" t="inlineStr"/>
+      <c r="W39" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3417,13 +3585,29 @@
           <t>Казань</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>kazan-hip.ru</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Казань (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr"/>
@@ -3433,7 +3617,9 @@
       <c r="T40" s="2" t="inlineStr"/>
       <c r="U40" s="2" t="inlineStr"/>
       <c r="V40" s="2" t="inlineStr"/>
-      <c r="W40" s="2" t="inlineStr"/>
+      <c r="W40" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3480,27 +3666,57 @@
           <t>Тюмень</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>jbi-5.ru</t>
+        </is>
+      </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Тюмень (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S41" s="2" t="inlineStr"/>
-      <c r="T41" s="2" t="inlineStr"/>
-      <c r="U41" s="2" t="inlineStr"/>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V41" s="2" t="inlineStr"/>
-      <c r="W41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3567,7 +3783,9 @@
       <c r="T42" s="2" t="inlineStr"/>
       <c r="U42" s="2" t="inlineStr"/>
       <c r="V42" s="2" t="inlineStr"/>
-      <c r="W42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3729,7 +3947,9 @@
       <c r="T44" s="2" t="inlineStr"/>
       <c r="U44" s="2" t="inlineStr"/>
       <c r="V44" s="2" t="inlineStr"/>
-      <c r="W44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -3796,7 +4016,9 @@
       <c r="T45" s="2" t="inlineStr"/>
       <c r="U45" s="2" t="inlineStr"/>
       <c r="V45" s="2" t="inlineStr"/>
-      <c r="W45" s="2" t="inlineStr"/>
+      <c r="W45" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -3855,7 +4077,9 @@
       <c r="T46" s="2" t="inlineStr"/>
       <c r="U46" s="2" t="inlineStr"/>
       <c r="V46" s="2" t="inlineStr"/>
-      <c r="W46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -3914,7 +4138,9 @@
       <c r="T47" s="2" t="inlineStr"/>
       <c r="U47" s="2" t="inlineStr"/>
       <c r="V47" s="2" t="inlineStr"/>
-      <c r="W47" s="2" t="inlineStr"/>
+      <c r="W47" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -3973,7 +4199,9 @@
       <c r="T48" s="2" t="inlineStr"/>
       <c r="U48" s="2" t="inlineStr"/>
       <c r="V48" s="2" t="inlineStr"/>
-      <c r="W48" s="2" t="inlineStr"/>
+      <c r="W48" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -4032,7 +4260,9 @@
       <c r="T49" s="2" t="inlineStr"/>
       <c r="U49" s="2" t="inlineStr"/>
       <c r="V49" s="2" t="inlineStr"/>
-      <c r="W49" s="2" t="inlineStr"/>
+      <c r="W49" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -4091,7 +4321,9 @@
       <c r="T50" s="2" t="inlineStr"/>
       <c r="U50" s="2" t="inlineStr"/>
       <c r="V50" s="2" t="inlineStr"/>
-      <c r="W50" s="2" t="inlineStr"/>
+      <c r="W50" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -4158,7 +4390,9 @@
       <c r="T51" s="2" t="inlineStr"/>
       <c r="U51" s="2" t="inlineStr"/>
       <c r="V51" s="2" t="inlineStr"/>
-      <c r="W51" s="2" t="inlineStr"/>
+      <c r="W51" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -4225,7 +4459,9 @@
       <c r="T52" s="2" t="inlineStr"/>
       <c r="U52" s="2" t="inlineStr"/>
       <c r="V52" s="2" t="inlineStr"/>
-      <c r="W52" s="2" t="inlineStr"/>
+      <c r="W52" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -4292,7 +4528,9 @@
       <c r="T53" s="2" t="inlineStr"/>
       <c r="U53" s="2" t="inlineStr"/>
       <c r="V53" s="2" t="inlineStr"/>
-      <c r="W53" s="2" t="inlineStr"/>
+      <c r="W53" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -4454,7 +4692,9 @@
       <c r="T55" s="2" t="inlineStr"/>
       <c r="U55" s="2" t="inlineStr"/>
       <c r="V55" s="2" t="inlineStr"/>
-      <c r="W55" s="2" t="inlineStr"/>
+      <c r="W55" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -4521,7 +4761,9 @@
       <c r="T56" s="2" t="inlineStr"/>
       <c r="U56" s="2" t="inlineStr"/>
       <c r="V56" s="2" t="inlineStr"/>
-      <c r="W56" s="2" t="inlineStr"/>
+      <c r="W56" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -4564,13 +4806,29 @@
           <t>Омск</t>
         </is>
       </c>
-      <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr"/>
-      <c r="M57" s="2" t="inlineStr"/>
-      <c r="N57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>gatp6omsk.ru</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 5506018844 найден на сайте</t>
+        </is>
+      </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr"/>
@@ -4580,7 +4838,9 @@
       <c r="T57" s="2" t="inlineStr"/>
       <c r="U57" s="2" t="inlineStr"/>
       <c r="V57" s="2" t="inlineStr"/>
-      <c r="W57" s="2" t="inlineStr"/>
+      <c r="W57" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -4623,23 +4883,57 @@
           <t>Екатеринбург</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr"/>
-      <c r="M58" s="2" t="inlineStr"/>
-      <c r="N58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>rodina-sk.ru</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Екатеринбург (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P58" s="2" t="inlineStr"/>
-      <c r="Q58" s="2" t="inlineStr"/>
-      <c r="R58" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S58" s="2" t="inlineStr"/>
-      <c r="T58" s="2" t="inlineStr"/>
-      <c r="U58" s="2" t="inlineStr"/>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V58" s="2" t="inlineStr"/>
-      <c r="W58" s="2" t="inlineStr"/>
+      <c r="W58" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -4686,27 +4980,61 @@
           <t>Воронеж</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>ladyanne-med.ru</t>
+        </is>
+      </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M59" s="2" t="inlineStr"/>
-      <c r="N59" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Воронеж (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P59" s="2" t="inlineStr"/>
-      <c r="Q59" s="2" t="inlineStr"/>
-      <c r="R59" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Расширенная консультация врача-косметолога и проведение 3D компьютерной диагностика кожи лица VISIA»</t>
+        </is>
+      </c>
       <c r="S59" s="2" t="inlineStr"/>
-      <c r="T59" s="2" t="inlineStr"/>
-      <c r="U59" s="2" t="inlineStr"/>
-      <c r="V59" s="2" t="inlineStr"/>
-      <c r="W59" s="2" t="inlineStr"/>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>похож</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>BBL Forever Clear Лицо (Лечение Акне), от; Расширенная консультация врача-косметолога и проведение 3D компьютерной диагностика кожи лица VISIA</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -4860,7 +5188,9 @@
       <c r="T61" s="2" t="inlineStr"/>
       <c r="U61" s="2" t="inlineStr"/>
       <c r="V61" s="2" t="inlineStr"/>
-      <c r="W61" s="2" t="inlineStr"/>
+      <c r="W61" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -4919,7 +5249,9 @@
       <c r="T62" s="2" t="inlineStr"/>
       <c r="U62" s="2" t="inlineStr"/>
       <c r="V62" s="2" t="inlineStr"/>
-      <c r="W62" s="2" t="inlineStr"/>
+      <c r="W62" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -4966,27 +5298,57 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>alstroyka.ru</t>
+        </is>
+      </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M63" s="2" t="inlineStr"/>
-      <c r="N63" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Самара (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P63" s="2" t="inlineStr"/>
-      <c r="Q63" s="2" t="inlineStr"/>
-      <c r="R63" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S63" s="2" t="inlineStr"/>
-      <c r="T63" s="2" t="inlineStr"/>
-      <c r="U63" s="2" t="inlineStr"/>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V63" s="2" t="inlineStr"/>
-      <c r="W63" s="2" t="inlineStr"/>
+      <c r="W63" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -5045,7 +5407,9 @@
       <c r="T64" s="2" t="inlineStr"/>
       <c r="U64" s="2" t="inlineStr"/>
       <c r="V64" s="2" t="inlineStr"/>
-      <c r="W64" s="2" t="inlineStr"/>
+      <c r="W64" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -5104,7 +5468,9 @@
       <c r="T65" s="2" t="inlineStr"/>
       <c r="U65" s="2" t="inlineStr"/>
       <c r="V65" s="2" t="inlineStr"/>
-      <c r="W65" s="2" t="inlineStr"/>
+      <c r="W65" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -5163,7 +5529,9 @@
       <c r="T66" s="2" t="inlineStr"/>
       <c r="U66" s="2" t="inlineStr"/>
       <c r="V66" s="2" t="inlineStr"/>
-      <c r="W66" s="2" t="inlineStr"/>
+      <c r="W66" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -5222,7 +5590,9 @@
       <c r="T67" s="2" t="inlineStr"/>
       <c r="U67" s="2" t="inlineStr"/>
       <c r="V67" s="2" t="inlineStr"/>
-      <c r="W67" s="2" t="inlineStr"/>
+      <c r="W67" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -5281,7 +5651,9 @@
       <c r="T68" s="2" t="inlineStr"/>
       <c r="U68" s="2" t="inlineStr"/>
       <c r="V68" s="2" t="inlineStr"/>
-      <c r="W68" s="2" t="inlineStr"/>
+      <c r="W68" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -5435,7 +5807,9 @@
       <c r="T70" s="2" t="inlineStr"/>
       <c r="U70" s="2" t="inlineStr"/>
       <c r="V70" s="2" t="inlineStr"/>
-      <c r="W70" s="2" t="inlineStr"/>
+      <c r="W70" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -5478,23 +5852,57 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr"/>
-      <c r="M71" s="2" t="inlineStr"/>
-      <c r="N71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>smr.center</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 6316281616 найден на сайте</t>
+        </is>
+      </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P71" s="2" t="inlineStr"/>
-      <c r="Q71" s="2" t="inlineStr"/>
-      <c r="R71" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Лицензия: Л041-01184-63/00660121 от 28.06.2023» (https://smr.center)</t>
+        </is>
+      </c>
       <c r="S71" s="2" t="inlineStr"/>
-      <c r="T71" s="2" t="inlineStr"/>
-      <c r="U71" s="2" t="inlineStr"/>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U71" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V71" s="2" t="inlineStr"/>
-      <c r="W71" s="2" t="inlineStr"/>
+      <c r="W71" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -5553,7 +5961,9 @@
       <c r="T72" s="2" t="inlineStr"/>
       <c r="U72" s="2" t="inlineStr"/>
       <c r="V72" s="2" t="inlineStr"/>
-      <c r="W72" s="2" t="inlineStr"/>
+      <c r="W72" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -5691,7 +6101,9 @@
       <c r="T74" s="2" t="inlineStr"/>
       <c r="U74" s="2" t="inlineStr"/>
       <c r="V74" s="2" t="inlineStr"/>
-      <c r="W74" s="2" t="inlineStr"/>
+      <c r="W74" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -5750,7 +6162,9 @@
       <c r="T75" s="2" t="inlineStr"/>
       <c r="U75" s="2" t="inlineStr"/>
       <c r="V75" s="2" t="inlineStr"/>
-      <c r="W75" s="2" t="inlineStr"/>
+      <c r="W75" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -5908,7 +6322,9 @@
       <c r="T77" s="2" t="inlineStr"/>
       <c r="U77" s="2" t="inlineStr"/>
       <c r="V77" s="2" t="inlineStr"/>
-      <c r="W77" s="2" t="inlineStr"/>
+      <c r="W77" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -5967,7 +6383,9 @@
       <c r="T78" s="2" t="inlineStr"/>
       <c r="U78" s="2" t="inlineStr"/>
       <c r="V78" s="2" t="inlineStr"/>
-      <c r="W78" s="2" t="inlineStr"/>
+      <c r="W78" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -6105,23 +6523,57 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="K80" s="2" t="inlineStr"/>
-      <c r="L80" s="2" t="inlineStr"/>
-      <c r="M80" s="2" t="inlineStr"/>
-      <c r="N80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>doctorermakov.ru</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Новосибирск (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P80" s="2" t="inlineStr"/>
-      <c r="Q80" s="2" t="inlineStr"/>
-      <c r="R80" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="R80" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Лицензия на осуществление медицинской деятельности № ЛО-54-01-005884» (https://doctorermakov.ru)</t>
+        </is>
+      </c>
       <c r="S80" s="2" t="inlineStr"/>
-      <c r="T80" s="2" t="inlineStr"/>
-      <c r="U80" s="2" t="inlineStr"/>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U80" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V80" s="2" t="inlineStr"/>
-      <c r="W80" s="2" t="inlineStr"/>
+      <c r="W80" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -6180,7 +6632,9 @@
       <c r="T81" s="2" t="inlineStr"/>
       <c r="U81" s="2" t="inlineStr"/>
       <c r="V81" s="2" t="inlineStr"/>
-      <c r="W81" s="2" t="inlineStr"/>
+      <c r="W81" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -6239,7 +6693,9 @@
       <c r="T82" s="2" t="inlineStr"/>
       <c r="U82" s="2" t="inlineStr"/>
       <c r="V82" s="2" t="inlineStr"/>
-      <c r="W82" s="2" t="inlineStr"/>
+      <c r="W82" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -6298,7 +6754,9 @@
       <c r="T83" s="2" t="inlineStr"/>
       <c r="U83" s="2" t="inlineStr"/>
       <c r="V83" s="2" t="inlineStr"/>
-      <c r="W83" s="2" t="inlineStr"/>
+      <c r="W83" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -6341,23 +6799,57 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr"/>
-      <c r="L84" s="2" t="inlineStr"/>
-      <c r="M84" s="2" t="inlineStr"/>
-      <c r="N84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>otkritie63.ru</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 6321384180 найден на сайте</t>
+        </is>
+      </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P84" s="2" t="inlineStr"/>
-      <c r="Q84" s="2" t="inlineStr"/>
-      <c r="R84" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R84" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S84" s="2" t="inlineStr"/>
-      <c r="T84" s="2" t="inlineStr"/>
-      <c r="U84" s="2" t="inlineStr"/>
+      <c r="T84" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U84" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V84" s="2" t="inlineStr"/>
-      <c r="W84" s="2" t="inlineStr"/>
+      <c r="W84" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -6416,7 +6908,9 @@
       <c r="T85" s="2" t="inlineStr"/>
       <c r="U85" s="2" t="inlineStr"/>
       <c r="V85" s="2" t="inlineStr"/>
-      <c r="W85" s="2" t="inlineStr"/>
+      <c r="W85" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -6483,7 +6977,9 @@
       <c r="T86" s="2" t="inlineStr"/>
       <c r="U86" s="2" t="inlineStr"/>
       <c r="V86" s="2" t="inlineStr"/>
-      <c r="W86" s="2" t="inlineStr"/>
+      <c r="W86" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -6550,7 +7046,9 @@
       <c r="T87" s="2" t="inlineStr"/>
       <c r="U87" s="2" t="inlineStr"/>
       <c r="V87" s="2" t="inlineStr"/>
-      <c r="W87" s="2" t="inlineStr"/>
+      <c r="W87" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -6617,7 +7115,9 @@
       <c r="T88" s="2" t="inlineStr"/>
       <c r="U88" s="2" t="inlineStr"/>
       <c r="V88" s="2" t="inlineStr"/>
-      <c r="W88" s="2" t="inlineStr"/>
+      <c r="W88" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -6660,23 +7160,57 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr"/>
-      <c r="M89" s="2" t="inlineStr"/>
-      <c r="N89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>xn----qtbcpidmcdj7fbs.xn--p1ai</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Новосибирск (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P89" s="2" t="inlineStr"/>
-      <c r="Q89" s="2" t="inlineStr"/>
-      <c r="R89" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R89" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S89" s="2" t="inlineStr"/>
-      <c r="T89" s="2" t="inlineStr"/>
-      <c r="U89" s="2" t="inlineStr"/>
+      <c r="T89" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="U89" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V89" s="2" t="inlineStr"/>
-      <c r="W89" s="2" t="inlineStr"/>
+      <c r="W89" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -6743,7 +7277,9 @@
       <c r="T90" s="2" t="inlineStr"/>
       <c r="U90" s="2" t="inlineStr"/>
       <c r="V90" s="2" t="inlineStr"/>
-      <c r="W90" s="2" t="inlineStr"/>
+      <c r="W90" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -6802,7 +7338,9 @@
       <c r="T91" s="2" t="inlineStr"/>
       <c r="U91" s="2" t="inlineStr"/>
       <c r="V91" s="2" t="inlineStr"/>
-      <c r="W91" s="2" t="inlineStr"/>
+      <c r="W91" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -6849,27 +7387,57 @@
           <t>Воронеж</t>
         </is>
       </c>
-      <c r="K92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>abireg.ru</t>
+        </is>
+      </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M92" s="2" t="inlineStr"/>
-      <c r="N92" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Воронеж (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P92" s="2" t="inlineStr"/>
-      <c r="Q92" s="2" t="inlineStr"/>
-      <c r="R92" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R92" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S92" s="2" t="inlineStr"/>
-      <c r="T92" s="2" t="inlineStr"/>
-      <c r="U92" s="2" t="inlineStr"/>
+      <c r="T92" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U92" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V92" s="2" t="inlineStr"/>
-      <c r="W92" s="2" t="inlineStr"/>
+      <c r="W92" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -6928,7 +7496,9 @@
       <c r="T93" s="2" t="inlineStr"/>
       <c r="U93" s="2" t="inlineStr"/>
       <c r="V93" s="2" t="inlineStr"/>
-      <c r="W93" s="2" t="inlineStr"/>
+      <c r="W93" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -6987,7 +7557,9 @@
       <c r="T94" s="2" t="inlineStr"/>
       <c r="U94" s="2" t="inlineStr"/>
       <c r="V94" s="2" t="inlineStr"/>
-      <c r="W94" s="2" t="inlineStr"/>
+      <c r="W94" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -7054,7 +7626,9 @@
       <c r="T95" s="2" t="inlineStr"/>
       <c r="U95" s="2" t="inlineStr"/>
       <c r="V95" s="2" t="inlineStr"/>
-      <c r="W95" s="2" t="inlineStr"/>
+      <c r="W95" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -7101,27 +7675,57 @@
           <t>Краснодар</t>
         </is>
       </c>
-      <c r="K96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>real-estetic.clients.site</t>
+        </is>
+      </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились</t>
-        </is>
-      </c>
-      <c r="M96" s="2" t="inlineStr"/>
-      <c r="N96" s="2" t="inlineStr"/>
+          <t>поиск (название+город)</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 2311160441 найден на сайте</t>
+        </is>
+      </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="P96" s="2" t="inlineStr"/>
-      <c r="Q96" s="2" t="inlineStr"/>
-      <c r="R96" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="R96" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="S96" s="2" t="inlineStr"/>
-      <c r="T96" s="2" t="inlineStr"/>
-      <c r="U96" s="2" t="inlineStr"/>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="U96" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V96" s="2" t="inlineStr"/>
-      <c r="W96" s="2" t="inlineStr"/>
+      <c r="W96" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -7188,7 +7792,9 @@
       <c r="T97" s="2" t="inlineStr"/>
       <c r="U97" s="2" t="inlineStr"/>
       <c r="V97" s="2" t="inlineStr"/>
-      <c r="W97" s="2" t="inlineStr"/>
+      <c r="W97" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -7247,7 +7853,9 @@
       <c r="T98" s="2" t="inlineStr"/>
       <c r="U98" s="2" t="inlineStr"/>
       <c r="V98" s="2" t="inlineStr"/>
-      <c r="W98" s="2" t="inlineStr"/>
+      <c r="W98" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -7306,7 +7914,9 @@
       <c r="T99" s="2" t="inlineStr"/>
       <c r="U99" s="2" t="inlineStr"/>
       <c r="V99" s="2" t="inlineStr"/>
-      <c r="W99" s="2" t="inlineStr"/>
+      <c r="W99" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -7365,7 +7975,9 @@
       <c r="T100" s="2" t="inlineStr"/>
       <c r="U100" s="2" t="inlineStr"/>
       <c r="V100" s="2" t="inlineStr"/>
-      <c r="W100" s="2" t="inlineStr"/>
+      <c r="W100" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -7519,7 +8131,9 @@
       <c r="T102" s="2" t="inlineStr"/>
       <c r="U102" s="2" t="inlineStr"/>
       <c r="V102" s="2" t="inlineStr"/>
-      <c r="W102" s="2" t="inlineStr"/>
+      <c r="W102" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -7578,7 +8192,9 @@
       <c r="T103" s="2" t="inlineStr"/>
       <c r="U103" s="2" t="inlineStr"/>
       <c r="V103" s="2" t="inlineStr"/>
-      <c r="W103" s="2" t="inlineStr"/>
+      <c r="W103" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -7637,7 +8253,9 @@
       <c r="T104" s="2" t="inlineStr"/>
       <c r="U104" s="2" t="inlineStr"/>
       <c r="V104" s="2" t="inlineStr"/>
-      <c r="W104" s="2" t="inlineStr"/>
+      <c r="W104" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -7696,7 +8314,9 @@
       <c r="T105" s="2" t="inlineStr"/>
       <c r="U105" s="2" t="inlineStr"/>
       <c r="V105" s="2" t="inlineStr"/>
-      <c r="W105" s="2" t="inlineStr"/>
+      <c r="W105" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -7755,7 +8375,9 @@
       <c r="T106" s="2" t="inlineStr"/>
       <c r="U106" s="2" t="inlineStr"/>
       <c r="V106" s="2" t="inlineStr"/>
-      <c r="W106" s="2" t="inlineStr"/>
+      <c r="W106" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -7822,7 +8444,9 @@
       <c r="T107" s="2" t="inlineStr"/>
       <c r="U107" s="2" t="inlineStr"/>
       <c r="V107" s="2" t="inlineStr"/>
-      <c r="W107" s="2" t="inlineStr"/>
+      <c r="W107" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -7881,7 +8505,9 @@
       <c r="T108" s="2" t="inlineStr"/>
       <c r="U108" s="2" t="inlineStr"/>
       <c r="V108" s="2" t="inlineStr"/>
-      <c r="W108" s="2" t="inlineStr"/>
+      <c r="W108" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -7940,7 +8566,9 @@
       <c r="T109" s="2" t="inlineStr"/>
       <c r="U109" s="2" t="inlineStr"/>
       <c r="V109" s="2" t="inlineStr"/>
-      <c r="W109" s="2" t="inlineStr"/>
+      <c r="W109" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7953,7 +8581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8004,26 +8632,26 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>1962</v>
+        <v>861</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>СТАНКОМАШ, ООО ИНДУСТРИАЛЬНЫЙ ПАРК</t>
+          <t>КЛИНИКИ НЕВРОЛОГИИ, ПСИХИАТРИИ И НАРКОЛОГИИ, ООО</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>7449059203</t>
+          <t>6316281616</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Челябинск</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>stankomash.konar.ru</t>
+          <t>smr.center</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -8033,32 +8661,32 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>лицензия (мед-контекст): «Лицензия № ЛО-74-01-005038 от 30.04.2019 г» (https://stankomash.konar.ru/uslugi)</t>
+          <t>лицензия (мед-контекст): «Лицензия: Л041-01184-63/00660121 от 28.06.2023» (https://smr.center)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>1987</v>
+        <v>999</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>СЦЛ, ООО</t>
+          <t>ЛЕДИ АННА ВРАЧЕБНО-КОСМЕТОЛОГИЧЕСКАЯ ЛЕЧЕБНИЦА, ООО</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2222841551</t>
+          <t>3666102811</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Барнаул</t>
+          <t>Воронеж</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>stomcenter22.ru</t>
+          <t>ladyanne-med.ru</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -8068,42 +8696,182 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>приём врача в прайсе: «Прием (осмотр, консультация) врача-стоматолога детского первичный»</t>
+          <t>приём врача в прайсе: «Расширенная консультация врача-косметолога и проведение 3D компьютерной диагностика кожи лица VISIA»</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
+        <v>1083</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>МЕДБИКО, ООО</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>5408307710</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>cnmt.ru</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Консультация флеболога и УЗИ вен за»</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>1962</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>СТАНКОМАШ, ООО ИНДУСТРИАЛЬНЫЙ ПАРК</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>7449059203</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Челябинск</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>stankomash.konar.ru</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Лицензия № ЛО-74-01-005038 от 30.04.2019 г» (https://stankomash.konar.ru/uslugi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>1987</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>СЦЛ, ООО</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2222841551</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Барнаул</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>stomcenter22.ru</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Прием (осмотр, консультация) врача-стоматолога детского первичный»</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>2115</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>ФРЕЙМ 4, ООО</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>6317157989</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Самара</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>frame4.ru</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>медорганизация</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>лицензия (мед-контекст): «Лицензия на осуществление медицинской деятельности № Л041-01184-63/00160045 от 06.05.2022 г» (https://frame4.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>2160</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ЦЕНТР ДОКТОРА ЕРМАКОВА, ООО</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>5406834694</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>doctorermakov.ru</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Лицензия на осуществление медицинской деятельности № ЛО-54-01-005884» (https://doctorermakov.ru)</t>
         </is>
       </c>
     </row>
@@ -8448,7 +9216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8499,26 +9267,26 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>354</v>
+        <v>107</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ГРУППА СИНАРА, АО</t>
+          <t>АЛЬЯНС, ООО</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>6658252583</t>
+          <t>6316050915</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>sinara-group.com</t>
+          <t>alstroyka.ru</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -8534,26 +9302,26 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>502</v>
+        <v>354</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ЗАПСИБГАЗПРОМ, ПАО</t>
+          <t>ГРУППА СИНАРА, АО</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>7203001796</t>
+          <t>6658252583</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Тюмень</t>
+          <t>Екатеринбург</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>zsgp.ru</t>
+          <t>sinara-group.com</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -8569,26 +9337,26 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>1115</v>
+        <v>499</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>МЕДИЦИНА И КАЧЕСТВО, ООО НПЦ ПКПС</t>
+          <t>ЗАВОД ЖБИ-5, АО ПРОМУЗЕЛ</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>6679075127</t>
+          <t>7203508145</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Тюмень</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>medkachestvo.ru</t>
+          <t>jbi-5.ru</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -8604,26 +9372,26 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>1578</v>
+        <v>502</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ОРДЖОНИКИДЗЕВСКАЯ УЖК, АО</t>
+          <t>ЗАПСИБГАЗПРОМ, ПАО</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>6673137722</t>
+          <t>7203001796</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Тюмень</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>ougk.ru</t>
+          <t>zsgp.ru</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -8639,26 +9407,26 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>1713</v>
+        <v>614</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ПРОФЕССИОНАЛ, ООО МК</t>
+          <t>КАРСАР, ООО</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>6311188074</t>
+          <t>1624004368</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Самара</t>
+          <t>Казань</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>mkprofessional63.ru</t>
+          <t>karsar.ru</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -8674,26 +9442,26 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>1854</v>
+        <v>676</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>СЕРВИС-БЕЗОПАСНОСТЬ, ООО</t>
+          <t>ККЗБ, ООО</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>3663095644</t>
+          <t>2311178167</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Воронеж</t>
+          <t>Краснодар</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>сервис-безопасность.рф</t>
+          <t>compressor-borec.ru</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8709,26 +9477,26 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>1977</v>
+        <v>1069</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>СТРОЙМЕХАНИЗАЦИЯ, АО</t>
+          <t>МЕБЕЛЬ ЧЕРНОЗЕМЬЯ, ООО ХК</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>5404109683</t>
+          <t>3661080681</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Новосибирск</t>
+          <t>Воронеж</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>oaosm-nsk.ru</t>
+          <t>abireg.ru</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -8744,34 +9512,384 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
+        <v>1115</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>МЕДИЦИНА И КАЧЕСТВО, ООО НПЦ ПКПС</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>6679075127</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>medkachestvo.ru</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>1231</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>МЕДЦЕНТР ОТКРЫТИЕ, ООО</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>6321384180</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Самара</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>otkritie63.ru</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>1578</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ОРДЖОНИКИДЗЕВСКАЯ УЖК, АО</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>6673137722</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ougk.ru</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>1593</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ОТКРЫТЫЙ ПУТЬ, ООО ЦЕНТР РАЗВИТИЯ</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>5404437821</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>xn----qtbcpidmcdj7fbs.xn--p1ai</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>1713</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ПРОФЕССИОНАЛ, ООО МК</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>6311188074</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Самара</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>mkprofessional63.ru</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>1789</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>РОДИНА, ООО СК</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>6685194490</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Екатеринбург</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>rodina-sk.ru</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>1820</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>САМСОН, ООО ПКФ</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2311004026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Краснодар</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>samson23.ru</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>1854</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>СЕРВИС-БЕЗОПАСНОСТЬ, ООО</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>3663095644</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Воронеж</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>сервис-безопасность.рф</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>1977</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>СТРОЙМЕХАНИЗАЦИЯ, АО</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>5404109683</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Новосибирск</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>oaosm-nsk.ru</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>2237</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>ЦЛМ РЕАЛ ЭСТЕТИК, ООО</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2311160441</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Краснодар</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>real-estetic.clients.site</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>2340</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>ЭНЕРГОМОНТАЖ, ООО</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>5410112902</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>em-nsk.ru</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>не определено</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
         </is>
@@ -8788,7 +9906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -9023,7 +10141,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
     </row>
@@ -9035,7 +10153,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -9047,7 +10165,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -9067,7 +10185,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>77</t>
         </is>
       </c>
     </row>
@@ -9079,7 +10197,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -9103,7 +10221,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -9123,7 +10241,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -9135,51 +10253,63 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>похож</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>— Стоимость —</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Поисковых запросов выполнено</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>— Стоимость —</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>Поисковых запросов выполнено</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>Потрачено, ₽ (0,52 ₽/запрос)</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>0.0</t>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>44.72</t>
         </is>
       </c>
     </row>

</xml_diff>